<commit_message>
docs(launch): clarify PostHog dashboard rollout
</commit_message>
<xml_diff>
--- a/docs/qa-matrix.xlsx
+++ b/docs/qa-matrix.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -574,7 +574,7 @@
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Region-aware hero ordering</t>
+          <t>Canadian-anchor hero</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -1005,7 +1005,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1034,12 +1034,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1054,21 +1054,17 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>Resend + Turnstile</t>
-        </is>
-      </c>
+      <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
@@ -1083,17 +1079,21 @@
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Turnstile-gated submit</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1110,19 +1110,19 @@
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Turnstile-gated submit</t>
+          <t>Lazy-imported surface</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
@@ -1139,19 +1139,19 @@
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Lazy-imported surface</t>
+          <t>PDF download</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1175,12 +1175,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
@@ -1197,19 +1197,19 @@
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>PDF download</t>
+          <t>Open + ask + cite + close</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
@@ -1224,36 +1224,7 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>Open + ask + cite + close</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1266,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F261"/>
+  <dimension ref="A1:F251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1502,7 +1473,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1702,7 +1673,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
@@ -1902,7 +1873,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -2102,7 +2073,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
@@ -2117,7 +2088,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2137,7 +2108,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2157,7 +2128,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2177,7 +2148,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2197,7 +2168,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2217,7 +2188,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2237,7 +2208,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2257,7 +2228,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2277,7 +2248,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2297,12 +2268,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Marketing — region-aware certs</t>
+          <t>Marketing — quality and compliance</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
@@ -2502,7 +2473,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -2702,7 +2673,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
@@ -2902,7 +2873,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr"/>
@@ -3102,7 +3073,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr"/>
@@ -3302,7 +3273,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr"/>
@@ -3502,7 +3473,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr"/>
@@ -3702,7 +3673,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr"/>
@@ -3902,7 +3873,7 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr"/>
@@ -4102,7 +4073,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr"/>
@@ -4302,7 +4273,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr"/>
@@ -4502,7 +4473,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr"/>
@@ -4702,7 +4673,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr"/>
@@ -4712,7 +4683,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -4732,7 +4703,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -4752,7 +4723,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -4772,7 +4743,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -4792,7 +4763,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -4812,7 +4783,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -4832,7 +4803,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -4852,7 +4823,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -4872,7 +4843,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -4892,7 +4863,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>/insights/del-at-a-glance-foreign-sponsor-primer</t>
+          <t>/insights/ich-q2-r2-method-validation-2024</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -4902,7 +4873,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr"/>
@@ -4912,12 +4883,12 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
@@ -4932,12 +4903,12 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
@@ -4952,12 +4923,12 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
@@ -4972,12 +4943,12 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
@@ -4992,12 +4963,12 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
@@ -5012,12 +4983,12 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
@@ -5032,12 +5003,12 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
@@ -5052,12 +5023,12 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
@@ -5072,12 +5043,12 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
@@ -5092,17 +5063,17 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>/insights/whitepapers/canadian-cdmo-operating-model</t>
+          <t>/our-process</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Whitepaper gate</t>
+          <t>Marketing — engagement workflow</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr"/>
@@ -5112,12 +5083,12 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
@@ -5132,12 +5103,12 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
@@ -5152,12 +5123,12 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
@@ -5172,12 +5143,12 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
@@ -5192,12 +5163,12 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
@@ -5212,12 +5183,12 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
@@ -5232,12 +5203,12 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
@@ -5252,12 +5223,12 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
@@ -5272,12 +5243,12 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
@@ -5292,17 +5263,17 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>/our-process</t>
+          <t>/contact</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>Marketing — engagement workflow</t>
+          <t>Form — inquiry + Cal.com + addresses</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr"/>
@@ -5312,12 +5283,12 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
@@ -5332,12 +5303,12 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
@@ -5352,12 +5323,12 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
@@ -5372,12 +5343,12 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
@@ -5392,12 +5363,12 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
@@ -5412,12 +5383,12 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
@@ -5432,12 +5403,12 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
@@ -5452,12 +5423,12 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
@@ -5472,12 +5443,12 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
@@ -5492,17 +5463,17 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>/contact</t>
+          <t>/ai/project-scoping-assistant</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Form — inquiry + Cal.com + addresses</t>
+          <t>AI tool — conversational scope</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr"/>
@@ -5512,12 +5483,12 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -5532,12 +5503,12 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -5552,12 +5523,12 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -5572,12 +5543,12 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
@@ -5592,12 +5563,12 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -5612,12 +5583,12 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
@@ -5632,12 +5603,12 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
@@ -5652,12 +5623,12 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -5672,12 +5643,12 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
@@ -5692,17 +5663,17 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>/ai/project-scoping-assistant</t>
+          <t>/ai/del-readiness</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>AI tool — conversational scope</t>
+          <t>AI tool — gap assessment</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr"/>
@@ -5712,12 +5683,12 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
@@ -5732,12 +5703,12 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
@@ -5752,12 +5723,12 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
@@ -5772,12 +5743,12 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
@@ -5792,12 +5763,12 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
@@ -5812,12 +5783,12 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
@@ -5832,12 +5803,12 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
@@ -5852,12 +5823,12 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
@@ -5872,12 +5843,12 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
@@ -5892,17 +5863,17 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>/ai/del-readiness</t>
+          <t>/ai/dosage-matcher</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>AI tool — gap assessment</t>
+          <t>AI tool — formulation match</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr"/>
@@ -5912,12 +5883,12 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
@@ -5932,12 +5903,12 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
@@ -5952,12 +5923,12 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
@@ -5972,12 +5943,12 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
@@ -5992,12 +5963,12 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
@@ -6012,12 +5983,12 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
@@ -6032,12 +6003,12 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -6052,12 +6023,12 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
@@ -6072,12 +6043,12 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -6092,17 +6063,17 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>/ai/dosage-matcher</t>
+          <t>(all)</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>AI tool — formulation match</t>
+          <t>Concierge bubble — site-wide</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr"/>
@@ -6112,12 +6083,12 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
@@ -6132,12 +6103,12 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -6152,12 +6123,12 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
@@ -6172,12 +6143,12 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
@@ -6192,12 +6163,12 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
@@ -6212,12 +6183,12 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
@@ -6232,12 +6203,12 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
@@ -6252,12 +6223,12 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
@@ -6272,12 +6243,12 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
@@ -6292,222 +6263,22 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>/accessibility</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Concierge bubble — site-wide</t>
+          <t>Statement</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Region cookie (px-region) does not break the page</t>
+          <t>No personalization cookie is required for the page to render correctly</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr"/>
       <c r="E251" s="2" t="inlineStr"/>
       <c r="F251" s="2" t="inlineStr"/>
-    </row>
-    <row r="252">
-      <c r="A252" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B252" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C252" s="2" t="inlineStr">
-        <is>
-          <t>Layout intact at the breakpoint (no overflow, no clipped text)</t>
-        </is>
-      </c>
-      <c r="D252" s="2" t="inlineStr"/>
-      <c r="E252" s="2" t="inlineStr"/>
-      <c r="F252" s="2" t="inlineStr"/>
-    </row>
-    <row r="253">
-      <c r="A253" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B253" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C253" s="2" t="inlineStr">
-        <is>
-          <t>All images load + have meaningful alt text where non-decorative</t>
-        </is>
-      </c>
-      <c r="D253" s="2" t="inlineStr"/>
-      <c r="E253" s="2" t="inlineStr"/>
-      <c r="F253" s="2" t="inlineStr"/>
-    </row>
-    <row r="254">
-      <c r="A254" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B254" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C254" s="2" t="inlineStr">
-        <is>
-          <t>Tab order follows visible order; visible focus ring on every interactive</t>
-        </is>
-      </c>
-      <c r="D254" s="2" t="inlineStr"/>
-      <c r="E254" s="2" t="inlineStr"/>
-      <c r="F254" s="2" t="inlineStr"/>
-    </row>
-    <row r="255">
-      <c r="A255" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B255" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C255" s="2" t="inlineStr">
-        <is>
-          <t>No console errors during initial paint or after interaction</t>
-        </is>
-      </c>
-      <c r="D255" s="2" t="inlineStr"/>
-      <c r="E255" s="2" t="inlineStr"/>
-      <c r="F255" s="2" t="inlineStr"/>
-    </row>
-    <row r="256">
-      <c r="A256" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B256" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C256" s="2" t="inlineStr">
-        <is>
-          <t>Primary CTA navigates to its declared destination</t>
-        </is>
-      </c>
-      <c r="D256" s="2" t="inlineStr"/>
-      <c r="E256" s="2" t="inlineStr"/>
-      <c r="F256" s="2" t="inlineStr"/>
-    </row>
-    <row r="257">
-      <c r="A257" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B257" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C257" s="2" t="inlineStr">
-        <is>
-          <t>Page passes the in-CI axe scan (zero serious or critical violations)</t>
-        </is>
-      </c>
-      <c r="D257" s="2" t="inlineStr"/>
-      <c r="E257" s="2" t="inlineStr"/>
-      <c r="F257" s="2" t="inlineStr"/>
-    </row>
-    <row r="258">
-      <c r="A258" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B258" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C258" s="2" t="inlineStr">
-        <is>
-          <t>Page meets the in-CI Lighthouse perf budget (warn at 0.90)</t>
-        </is>
-      </c>
-      <c r="D258" s="2" t="inlineStr"/>
-      <c r="E258" s="2" t="inlineStr"/>
-      <c r="F258" s="2" t="inlineStr"/>
-    </row>
-    <row r="259">
-      <c r="A259" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B259" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C259" s="2" t="inlineStr">
-        <is>
-          <t>JSON-LD validates in Schema.org Validator</t>
-        </is>
-      </c>
-      <c r="D259" s="2" t="inlineStr"/>
-      <c r="E259" s="2" t="inlineStr"/>
-      <c r="F259" s="2" t="inlineStr"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B260" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C260" s="2" t="inlineStr">
-        <is>
-          <t>OG tags render correctly when previewed in social-link debugger</t>
-        </is>
-      </c>
-      <c r="D260" s="2" t="inlineStr"/>
-      <c r="E260" s="2" t="inlineStr"/>
-      <c r="F260" s="2" t="inlineStr"/>
-    </row>
-    <row r="261">
-      <c r="A261" s="2" t="inlineStr">
-        <is>
-          <t>/accessibility</t>
-        </is>
-      </c>
-      <c r="B261" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="C261" s="2" t="inlineStr">
-        <is>
-          <t>Region cookie (px-region) does not break the page</t>
-        </is>
-      </c>
-      <c r="D261" s="2" t="inlineStr"/>
-      <c r="E261" s="2" t="inlineStr"/>
-      <c r="F261" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6593,7 +6364,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bundle budget (450 kB) green per .github/workflows/bundle-budget.yml</t>
+          <t>Bundle budget (350 kB) green per .github/workflows/bundle-budget.yml</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -6648,7 +6419,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PostHog dashboards live (per docs/analytics-taxonomy.md §6)</t>
+          <t>PostHog dashboards live (per docs/posthog-dashboard-build-sheet.md)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>

</xml_diff>